<commit_message>
fix: remove quote and use new format for quotation, delivery note and tax invoice
</commit_message>
<xml_diff>
--- a/templates/documents/quotation.xlsx
+++ b/templates/documents/quotation.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
-  <si>
-    <t>DEEZANO</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>DEEZANO CLOTHING LINE LLC</t>
   </si>
   <si>
     <t>TRN:104067685800003</t>
@@ -41,6 +41,9 @@
   </si>
   <si>
     <t>CUSTOMER</t>
+  </si>
+  <si>
+    <t>VALIDITY#</t>
   </si>
   <si>
     <t>NO.</t>
@@ -78,7 +81,7 @@
         <sz val="6"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>QANTITY</t>
+      <t>QUANTITY</t>
     </r>
   </si>
   <si>
@@ -115,17 +118,27 @@
     <t>GRAND TOTAL</t>
   </si>
   <si>
-    <t>DEEZANO CLOTHING LINE LLC , 971502641611 , info@deezanoae.com</t>
+    <t>TERMS AND CONDITIONS</t>
+  </si>
+  <si>
+    <t>Term text</t>
+  </si>
+  <si>
+    <t>DEEZANO CLOTHING LINE LLC , 971502641611 , info@deezanoapparel.com</t>
+  </si>
+  <si>
+    <t>DUBAI, UAE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0_);(0)"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="31" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -145,12 +158,6 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <color theme="1"/>
-      <family val="2"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <u/>
       <family val="2"/>
       <sz val="9"/>
@@ -215,10 +222,9 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
       <color theme="1"/>
       <family val="2"/>
-      <sz val="9"/>
+      <sz val="12"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -235,12 +241,6 @@
       <name val="Trebuchet MS"/>
     </font>
     <font>
-      <color rgb="FF000000"/>
-      <family val="2"/>
-      <sz val="6"/>
-      <name val="Trebuchet MS"/>
-    </font>
-    <font>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="9"/>
@@ -296,15 +296,16 @@
     </font>
     <font>
       <b/>
-      <color theme="1"/>
-      <family val="2"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF101010"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+      <name val="Trebuchet MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Trebuchet MS"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Trebuchet MS"/>
     </font>
@@ -387,7 +388,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1" indent="4"/>
@@ -395,164 +396,145 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="23" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="21" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="23" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="21" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="23" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="23" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="24" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="25" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="25" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="26" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -577,11 +559,11 @@
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>12700</xdr:colOff>
+      <xdr:colOff>12800</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>22860</xdr:rowOff>
+      <xdr:rowOff>17500</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1788159" cy="385798"/>
+    <xdr:ext cx="1524000" cy="619125"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -846,24 +828,25 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:Q26"/>
+  <dimension ref="B2:G30"/>
   <sheetFormatPr defaultRowHeight="13" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.15" customHeight="1"/>
   <cols>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="48.796875" customWidth="1"/>
-    <col min="6" max="6" width="16.59765625" customWidth="1"/>
-    <col min="7" max="7" width="22.3984375" customWidth="1"/>
+    <col min="2" max="2" width="13.3" customWidth="1"/>
+    <col min="3" max="3" width="11.7" customWidth="1"/>
+    <col min="4" max="4" width="48.8" customWidth="1"/>
+    <col min="5" max="5" width="12.7" customWidth="1"/>
+    <col min="6" max="6" width="16.7" customWidth="1"/>
+    <col min="7" max="7" width="22.4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="35" customHeight="1" spans="3:8" x14ac:dyDescent="0.25">
+    <row r="2" ht="54" customHeight="1" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-    </row>
-    <row r="3" ht="16" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
@@ -872,285 +855,242 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="3"/>
-    </row>
-    <row r="4" ht="16" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="3"/>
-    </row>
-    <row r="5" ht="19" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="5">
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" ht="19" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="4">
         <v>971502641611</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="3"/>
-    </row>
-    <row r="6" ht="21" customHeight="1" spans="2:8" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="8" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+    </row>
+    <row r="6" ht="21" customHeight="1" spans="2:7" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="11" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="11"/>
-      <c r="H6" s="12"/>
-    </row>
-    <row r="7" ht="16" customHeight="1" spans="2:8" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G6" s="10"/>
+    </row>
+    <row r="7" ht="16" customHeight="1" spans="2:7" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="12"/>
-    </row>
-    <row r="8" ht="16" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="15" t="s">
+      <c r="E7" s="11"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+    </row>
+    <row r="8" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="16" t="s">
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="G8" s="17"/>
-      <c r="H8" s="12"/>
-    </row>
-    <row r="9" ht="16" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="18"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="21" t="s">
+      <c r="G8" s="15"/>
+    </row>
+    <row r="9" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="16"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="G9" s="17"/>
-      <c r="H9" s="12"/>
-    </row>
-    <row r="10" ht="16" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="22" t="s">
+      <c r="G9" s="15"/>
+    </row>
+    <row r="10" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="12"/>
-    </row>
-    <row r="11" ht="16" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="12"/>
-    </row>
-    <row r="12" ht="16" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="12"/>
-    </row>
-    <row r="13" ht="16" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="12"/>
-      <c r="L13" s="29"/>
-      <c r="M13" s="29"/>
-    </row>
-    <row r="14" ht="16" customHeight="1" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="30"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="12"/>
-      <c r="L14" s="29"/>
-      <c r="M14" s="29"/>
-    </row>
-    <row r="15" ht="16" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" s="15"/>
+    </row>
+    <row r="11" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="24"/>
+    </row>
+    <row r="12" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="21"/>
+    </row>
+    <row r="13" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="25"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="21"/>
+    </row>
+    <row r="14" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="27"/>
+    </row>
+    <row r="15" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="12"/>
-    </row>
-    <row r="16" ht="16" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="12"/>
-    </row>
-    <row r="17" ht="16" customHeight="1" spans="2:17" s="33" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="34" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="35" t="s">
+      <c r="G15" s="18"/>
+    </row>
+    <row r="16" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+    </row>
+    <row r="17" ht="16" customHeight="1" spans="2:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="35" t="s">
+      <c r="C17" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="35" t="s">
+      <c r="D17" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="F17" s="35" t="s">
+      <c r="E17" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="35" t="s">
+      <c r="F17" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="H17" s="36"/>
-      <c r="I17" s="33"/>
-      <c r="J17" s="33"/>
-      <c r="K17" s="33"/>
-      <c r="L17" s="33"/>
-      <c r="M17" s="33"/>
-      <c r="N17" s="33"/>
-      <c r="O17" s="33"/>
-      <c r="P17" s="33"/>
-      <c r="Q17" s="33"/>
-    </row>
-    <row r="18" ht="48" customHeight="1" spans="2:17" s="37" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="38"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="43"/>
-      <c r="I18" s="37"/>
-      <c r="J18" s="37"/>
-      <c r="K18" s="37"/>
-      <c r="L18" s="37"/>
-      <c r="M18" s="37"/>
-      <c r="N18" s="37"/>
-      <c r="O18" s="37"/>
-      <c r="P18" s="37"/>
-      <c r="Q18" s="37"/>
-    </row>
-    <row r="19" ht="48" customHeight="1" spans="2:8" s="37" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="38"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="40"/>
-      <c r="E19" s="41"/>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="43"/>
-    </row>
-    <row r="20" ht="16" customHeight="1" spans="2:17" s="33" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="44"/>
-      <c r="C20" s="45" t="s">
+      <c r="G17" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="45"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="45"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="36"/>
-      <c r="I20" s="47"/>
-      <c r="J20" s="47"/>
-      <c r="K20" s="47"/>
-      <c r="L20" s="47"/>
-      <c r="M20" s="47"/>
-      <c r="N20" s="47"/>
-      <c r="O20" s="47"/>
-      <c r="P20" s="47"/>
-      <c r="Q20" s="47"/>
-    </row>
-    <row r="21" ht="16" customHeight="1" spans="2:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="44"/>
-      <c r="C21" s="48" t="s">
+    </row>
+    <row r="18" ht="48" customHeight="1" spans="2:7" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="33"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+    </row>
+    <row r="19" ht="48" customHeight="1" spans="2:7" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="33"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="37"/>
+      <c r="G19" s="37"/>
+    </row>
+    <row r="20" ht="16" customHeight="1" spans="2:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="38"/>
+      <c r="C20" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="D21" s="48"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="48"/>
-      <c r="G21" s="49"/>
-      <c r="H21" s="36"/>
-    </row>
-    <row r="22" ht="16" customHeight="1" spans="2:8" s="33" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="44"/>
-      <c r="C22" s="48" t="s">
+      <c r="D20" s="39"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="40"/>
+    </row>
+    <row r="21" ht="16" customHeight="1" spans="2:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="38"/>
+      <c r="C21" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="D22" s="48"/>
-      <c r="E22" s="48"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="50"/>
-      <c r="H22" s="36"/>
-    </row>
-    <row r="23" ht="16" customHeight="1" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="51"/>
-      <c r="H23" s="12"/>
-    </row>
-    <row r="24" ht="16" customHeight="1" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C24" s="52"/>
-      <c r="D24" s="53"/>
-      <c r="E24" s="53"/>
-      <c r="F24" s="53"/>
-      <c r="G24" s="53"/>
-      <c r="H24" s="53"/>
-    </row>
-    <row r="25" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C25" s="54" t="s">
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="42"/>
+    </row>
+    <row r="22" ht="16" customHeight="1" spans="2:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="38"/>
+      <c r="C22" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="D25" s="54"/>
-      <c r="E25" s="54"/>
-      <c r="F25" s="54"/>
-      <c r="G25" s="54"/>
-      <c r="H25" s="54"/>
-    </row>
-    <row r="26" ht="16" customHeight="1" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="C26" s="55" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" s="55"/>
-      <c r="E26" s="55"/>
-      <c r="F26" s="55"/>
-      <c r="G26" s="55"/>
-      <c r="H26" s="55"/>
-    </row>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="43"/>
+    </row>
+    <row r="23" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="18" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="44"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="44"/>
+    </row>
+    <row r="25" ht="40" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B25" s="45">
+        <v>1</v>
+      </c>
+      <c r="C25" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25"/>
+      <c r="E25"/>
+      <c r="F25"/>
+    </row>
+    <row r="26" ht="16" customHeight="1" spans="2:7" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="18" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28"/>
+      <c r="D28"/>
+      <c r="E28"/>
+      <c r="F28"/>
+    </row>
+    <row r="29" ht="18" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29"/>
+      <c r="D29"/>
+      <c r="E29"/>
+      <c r="F29"/>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="C2:H2"/>
+  <mergeCells count="22">
+    <mergeCell ref="C2:G2"/>
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B5:D5"/>
@@ -1163,24 +1103,21 @@
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
-    <mergeCell ref="L13:M14"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B15:D15"/>
-    <mergeCell ref="I17:Q17"/>
-    <mergeCell ref="I18:Q18"/>
     <mergeCell ref="C20:F20"/>
-    <mergeCell ref="I20:Q20"/>
     <mergeCell ref="C21:F21"/>
     <mergeCell ref="C22:F22"/>
-    <mergeCell ref="D24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B6" r:id="rId1"/>
   </hyperlinks>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" scale="45" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>